<commit_message>
Excluir subcontenidos de Licencias y Vehiculos SAP del top 10
- Capa 2: agrega MO08CUX03 Apertura (sub de Trámites Vehículos SAP, ene-2026 puesto 10)
- Capa 2: agrega Licencia prorroga > Consultar, MO05CUX01 > Tiene que renovar, LIC00CUX00 Validaciones (subs de Licencias, feb-2026 puestos 9 y 10)
- Capa 1: agrega patrón BOT0
- Crea exclusiones_capa2.md con registro completo de todo lo excluido (Capa 1 y Capa 2)
- Regenera outputs de febrero 2026

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Contenidos_Consultados/output/contenidos_consultados_febrero_2026.xlsx
+++ b/Contenidos_Consultados/output/contenidos_consultados_febrero_2026.xlsx
@@ -582,16 +582,16 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>1- SA06CUX03 Confirmar turno Sí, dale: (373.253)
-2- miBA - Login exitoso: (144.056)
-3- TUR00CUX02 Turnos para salud: (133.598)
-4- Infracciones * Apertura: (125.263)
-5- SA06CUX02 Apertura: (100.459)
-6- MO00CUX01 Auto o moto: (95.631)
-7- SA10CUX01 Hospitales: (75.067)
-8- MO05CUX02 Apertura: (72.302)
-9- TR00CUX01 Apertura: (62.913)
-10- Licencia prorroga  &gt; Consultar: (62.240)</t>
+          <t>1- Confirmación Turnos Salud: (373.253)
+2- Turnos Salud: (133.598)
+3- Infracciones: (125.263)
+4- Mis profesionales: (100.459)
+5- Trámites Vehículos SAP: (95.631)
+6- Hospitales: (75.067)
+7- Licencias: (72.302)
+8- Trámites SAP: (62.913)
+9- Buscar donde está permitido estacionar: (47.309)
+10- SA17CUX01 Apertura : (26.026)</t>
         </is>
       </c>
     </row>

</xml_diff>